<commit_message>
Update eclat_habitos_compra notebook with new Markdown structure, enhancing documentation and clarity. Added new cells for code execution and defined global parameters. Replace df_procesado.xlsx and dataset.xlsx with updated versions for improved data handling.
</commit_message>
<xml_diff>
--- a/data/dataset.xlsx
+++ b/data/dataset.xlsx
@@ -8,19 +8,31 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Todo\Descargas\Mineria\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A23FD186-2C9E-4229-8DDE-9058E5AC7B9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08E0358A-12E5-4443-A415-B6DCACEF587B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20640" windowHeight="11760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Respuestas de formulario 1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3034" uniqueCount="1095">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3034" uniqueCount="1097">
   <si>
     <t>Marca temporal</t>
   </si>
@@ -3788,6 +3800,12 @@
   </si>
   <si>
     <t>frijoles, chocolate, sal, acondicionador, harinas, crema dental, carne de res, galletas</t>
+  </si>
+  <si>
+    <t>Boyaca</t>
+  </si>
+  <si>
+    <t>Pereira</t>
   </si>
 </sst>
 </file>
@@ -5522,7 +5540,7 @@
         <v>20</v>
       </c>
       <c r="E24" t="s">
-        <v>45</v>
+        <v>128</v>
       </c>
       <c r="F24" t="s">
         <v>22</v>
@@ -5640,7 +5658,7 @@
         <v>34</v>
       </c>
       <c r="E26" t="s">
-        <v>45</v>
+        <v>128</v>
       </c>
       <c r="F26" t="s">
         <v>22</v>
@@ -5817,7 +5835,7 @@
         <v>135</v>
       </c>
       <c r="E29" t="s">
-        <v>45</v>
+        <v>128</v>
       </c>
       <c r="F29" t="s">
         <v>22</v>
@@ -5876,7 +5894,7 @@
         <v>135</v>
       </c>
       <c r="E30" t="s">
-        <v>185</v>
+        <v>128</v>
       </c>
       <c r="F30" t="s">
         <v>55</v>
@@ -6171,7 +6189,7 @@
         <v>34</v>
       </c>
       <c r="E35" t="s">
-        <v>35</v>
+        <v>128</v>
       </c>
       <c r="F35" t="s">
         <v>55</v>
@@ -6348,7 +6366,7 @@
         <v>184</v>
       </c>
       <c r="E38" t="s">
-        <v>285</v>
+        <v>128</v>
       </c>
       <c r="F38" t="s">
         <v>55</v>
@@ -6525,7 +6543,7 @@
         <v>135</v>
       </c>
       <c r="E41" t="s">
-        <v>80</v>
+        <v>128</v>
       </c>
       <c r="F41" t="s">
         <v>22</v>
@@ -6820,7 +6838,7 @@
         <v>34</v>
       </c>
       <c r="E46" t="s">
-        <v>35</v>
+        <v>128</v>
       </c>
       <c r="F46" t="s">
         <v>22</v>
@@ -6879,7 +6897,7 @@
         <v>135</v>
       </c>
       <c r="E47" t="s">
-        <v>35</v>
+        <v>128</v>
       </c>
       <c r="F47" t="s">
         <v>22</v>
@@ -7174,7 +7192,7 @@
         <v>135</v>
       </c>
       <c r="E52" t="s">
-        <v>80</v>
+        <v>1095</v>
       </c>
       <c r="F52" t="s">
         <v>55</v>
@@ -7410,7 +7428,7 @@
         <v>20</v>
       </c>
       <c r="E56" t="s">
-        <v>45</v>
+        <v>1095</v>
       </c>
       <c r="F56" t="s">
         <v>55</v>
@@ -7469,7 +7487,7 @@
         <v>34</v>
       </c>
       <c r="E57" t="s">
-        <v>71</v>
+        <v>1095</v>
       </c>
       <c r="F57" t="s">
         <v>55</v>
@@ -7882,7 +7900,7 @@
         <v>135</v>
       </c>
       <c r="E64" t="s">
-        <v>45</v>
+        <v>1095</v>
       </c>
       <c r="F64" t="s">
         <v>22</v>
@@ -7941,7 +7959,7 @@
         <v>135</v>
       </c>
       <c r="E65" t="s">
-        <v>285</v>
+        <v>1095</v>
       </c>
       <c r="F65" t="s">
         <v>55</v>
@@ -8000,7 +8018,7 @@
         <v>34</v>
       </c>
       <c r="E66" t="s">
-        <v>21</v>
+        <v>1095</v>
       </c>
       <c r="F66" t="s">
         <v>22</v>
@@ -8177,7 +8195,7 @@
         <v>34</v>
       </c>
       <c r="E69" t="s">
-        <v>45</v>
+        <v>1096</v>
       </c>
       <c r="F69" t="s">
         <v>22</v>
@@ -8413,7 +8431,7 @@
         <v>135</v>
       </c>
       <c r="E73" t="s">
-        <v>163</v>
+        <v>1095</v>
       </c>
       <c r="F73" t="s">
         <v>22</v>
@@ -8472,7 +8490,7 @@
         <v>135</v>
       </c>
       <c r="E74" t="s">
-        <v>45</v>
+        <v>1095</v>
       </c>
       <c r="F74" t="s">
         <v>22</v>
@@ -8590,7 +8608,7 @@
         <v>20</v>
       </c>
       <c r="E76" t="s">
-        <v>185</v>
+        <v>1096</v>
       </c>
       <c r="F76" t="s">
         <v>55</v>
@@ -8649,7 +8667,7 @@
         <v>20</v>
       </c>
       <c r="E77" t="s">
-        <v>285</v>
+        <v>128</v>
       </c>
       <c r="F77" t="s">
         <v>55</v>
@@ -8767,7 +8785,7 @@
         <v>34</v>
       </c>
       <c r="E79" t="s">
-        <v>185</v>
+        <v>1096</v>
       </c>
       <c r="F79" t="s">
         <v>55</v>
@@ -8944,7 +8962,7 @@
         <v>20</v>
       </c>
       <c r="E82" t="s">
-        <v>80</v>
+        <v>1096</v>
       </c>
       <c r="F82" t="s">
         <v>22</v>
@@ -9180,7 +9198,7 @@
         <v>20</v>
       </c>
       <c r="E86" t="s">
-        <v>35</v>
+        <v>21</v>
       </c>
       <c r="F86" t="s">
         <v>22</v>
@@ -9298,7 +9316,7 @@
         <v>20</v>
       </c>
       <c r="E88" t="s">
-        <v>35</v>
+        <v>21</v>
       </c>
       <c r="F88" t="s">
         <v>55</v>
@@ -9357,7 +9375,7 @@
         <v>20</v>
       </c>
       <c r="E89" t="s">
-        <v>35</v>
+        <v>21</v>
       </c>
       <c r="F89" t="s">
         <v>22</v>
@@ -9416,7 +9434,7 @@
         <v>34</v>
       </c>
       <c r="E90" t="s">
-        <v>45</v>
+        <v>21</v>
       </c>
       <c r="F90" t="s">
         <v>55</v>
@@ -9711,7 +9729,7 @@
         <v>20</v>
       </c>
       <c r="E95" t="s">
-        <v>35</v>
+        <v>21</v>
       </c>
       <c r="F95" t="s">
         <v>22</v>
@@ -9770,7 +9788,7 @@
         <v>20</v>
       </c>
       <c r="E96" t="s">
-        <v>35</v>
+        <v>21</v>
       </c>
       <c r="F96" t="s">
         <v>55</v>
@@ -9829,7 +9847,7 @@
         <v>20</v>
       </c>
       <c r="E97" t="s">
-        <v>357</v>
+        <v>21</v>
       </c>
       <c r="F97" t="s">
         <v>55</v>
@@ -9947,7 +9965,7 @@
         <v>34</v>
       </c>
       <c r="E99" t="s">
-        <v>35</v>
+        <v>21</v>
       </c>
       <c r="F99" t="s">
         <v>55</v>
@@ -10065,7 +10083,7 @@
         <v>135</v>
       </c>
       <c r="E101" t="s">
-        <v>163</v>
+        <v>21</v>
       </c>
       <c r="F101" t="s">
         <v>22</v>
@@ -10938,7 +10956,7 @@
     </row>
     <row r="116" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A116" s="1">
-        <v>46137.432638888888</v>
+        <v>46129.432638888888</v>
       </c>
       <c r="B116">
         <v>19</v>
@@ -10997,7 +11015,7 @@
     </row>
     <row r="117" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A117" s="1">
-        <v>46137.520833333343</v>
+        <v>46133.208634259259</v>
       </c>
       <c r="B117">
         <v>20</v>
@@ -11056,7 +11074,7 @@
     </row>
     <row r="118" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A118" s="1">
-        <v>46137.579861111109</v>
+        <v>46133.031423611108</v>
       </c>
       <c r="B118">
         <v>22</v>
@@ -11115,7 +11133,7 @@
     </row>
     <row r="119" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A119" s="1">
-        <v>46137.770833333343</v>
+        <v>46129.342893518522</v>
       </c>
       <c r="B119">
         <v>21</v>
@@ -11174,7 +11192,7 @@
     </row>
     <row r="120" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A120" s="1">
-        <v>46137.956250000003</v>
+        <v>46126.909236111111</v>
       </c>
       <c r="B120">
         <v>21</v>
@@ -11233,7 +11251,7 @@
     </row>
     <row r="121" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A121" s="1">
-        <v>46138.329861111109</v>
+        <v>46132.700902777775</v>
       </c>
       <c r="B121">
         <v>21</v>
@@ -11292,7 +11310,7 @@
     </row>
     <row r="122" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A122" s="1">
-        <v>46138.379166666673</v>
+        <v>46131.385034722225</v>
       </c>
       <c r="B122">
         <v>24</v>
@@ -11351,7 +11369,7 @@
     </row>
     <row r="123" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A123" s="1">
-        <v>46138.443749999999</v>
+        <v>46128.446226851855</v>
       </c>
       <c r="B123">
         <v>18</v>
@@ -11410,7 +11428,7 @@
     </row>
     <row r="124" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A124" s="1">
-        <v>46138.677083333343</v>
+        <v>46125.624918981484</v>
       </c>
       <c r="B124">
         <v>19</v>
@@ -11469,7 +11487,7 @@
     </row>
     <row r="125" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A125" s="1">
-        <v>46138.743750000001</v>
+        <v>46130.389085648145</v>
       </c>
       <c r="B125">
         <v>21</v>
@@ -11528,7 +11546,7 @@
     </row>
     <row r="126" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A126" s="1">
-        <v>46139.321527777778</v>
+        <v>46130.067476851851</v>
       </c>
       <c r="B126">
         <v>21</v>
@@ -11587,7 +11605,7 @@
     </row>
     <row r="127" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A127" s="1">
-        <v>46139.481944444437</v>
+        <v>46132.506608796299</v>
       </c>
       <c r="B127">
         <v>20</v>
@@ -11646,7 +11664,7 @@
     </row>
     <row r="128" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A128" s="1">
-        <v>46139.70416666667</v>
+        <v>46125.227905092594</v>
       </c>
       <c r="B128">
         <v>20</v>
@@ -11705,7 +11723,7 @@
     </row>
     <row r="129" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A129" s="1">
-        <v>46139.736805555563</v>
+        <v>46132.365914351853</v>
       </c>
       <c r="B129">
         <v>20</v>
@@ -11764,7 +11782,7 @@
     </row>
     <row r="130" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A130" s="1">
-        <v>46139.884027777778</v>
+        <v>46125.518425925926</v>
       </c>
       <c r="B130">
         <v>24</v>
@@ -11823,7 +11841,7 @@
     </row>
     <row r="131" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A131" s="1">
-        <v>46140.318055555559</v>
+        <v>46127.137430555558</v>
       </c>
       <c r="B131">
         <v>21</v>
@@ -11882,7 +11900,7 @@
     </row>
     <row r="132" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A132" s="1">
-        <v>46140.494444444441</v>
+        <v>46128.105150462965</v>
       </c>
       <c r="B132">
         <v>22</v>
@@ -11941,7 +11959,7 @@
     </row>
     <row r="133" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A133" s="1">
-        <v>46140.692361111112</v>
+        <v>46128.933611111112</v>
       </c>
       <c r="B133">
         <v>25</v>
@@ -12000,7 +12018,7 @@
     </row>
     <row r="134" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A134" s="1">
-        <v>46140.791666666657</v>
+        <v>46129.508645833332</v>
       </c>
       <c r="B134">
         <v>21</v>
@@ -12059,7 +12077,7 @@
     </row>
     <row r="135" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A135" s="1">
-        <v>46141.321527777778</v>
+        <v>46131.69121527778</v>
       </c>
       <c r="B135">
         <v>20</v>
@@ -12118,7 +12136,7 @@
     </row>
     <row r="136" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A136" s="1">
-        <v>46141.588194444441</v>
+        <v>46131.723032407404</v>
       </c>
       <c r="B136">
         <v>21</v>
@@ -12177,7 +12195,7 @@
     </row>
     <row r="137" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A137" s="1">
-        <v>46141.638888888891</v>
+        <v>46130.376701388886</v>
       </c>
       <c r="B137">
         <v>22</v>
@@ -12236,7 +12254,7 @@
     </row>
     <row r="138" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A138" s="1">
-        <v>46141.89166666667</v>
+        <v>46133.699201388888</v>
       </c>
       <c r="B138">
         <v>20</v>
@@ -12295,7 +12313,7 @@
     </row>
     <row r="139" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A139" s="1">
-        <v>46142.324999999997</v>
+        <v>46126.180011574077</v>
       </c>
       <c r="B139">
         <v>20</v>
@@ -12354,7 +12372,7 @@
     </row>
     <row r="140" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A140" s="1">
-        <v>46142.429861111108</v>
+        <v>46128.94494212963</v>
       </c>
       <c r="B140">
         <v>18</v>
@@ -12413,7 +12431,7 @@
     </row>
     <row r="141" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A141" s="1">
-        <v>46142.713194444441</v>
+        <v>46130.629537037035</v>
       </c>
       <c r="B141">
         <v>19</v>
@@ -12472,7 +12490,7 @@
     </row>
     <row r="142" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A142" s="1">
-        <v>46142.951388888891</v>
+        <v>46132.953287037039</v>
       </c>
       <c r="B142">
         <v>20</v>
@@ -12531,7 +12549,7 @@
     </row>
     <row r="143" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A143" s="1">
-        <v>46143.296527777777</v>
+        <v>46125.386365740742</v>
       </c>
       <c r="B143">
         <v>21</v>
@@ -12590,7 +12608,7 @@
     </row>
     <row r="144" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A144" s="1">
-        <v>46143.411111111112</v>
+        <v>46133.219641203701</v>
       </c>
       <c r="B144">
         <v>20</v>
@@ -12649,7 +12667,7 @@
     </row>
     <row r="145" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A145" s="1">
-        <v>46143.575694444437</v>
+        <v>46128.730393518519</v>
       </c>
       <c r="B145">
         <v>20</v>
@@ -12708,7 +12726,7 @@
     </row>
     <row r="146" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A146" s="1">
-        <v>46143.64166666667</v>
+        <v>46128.358275462961</v>
       </c>
       <c r="B146">
         <v>22</v>
@@ -12767,7 +12785,7 @@
     </row>
     <row r="147" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A147" s="1">
-        <v>46143.813194444447</v>
+        <v>46126.608784722222</v>
       </c>
       <c r="B147">
         <v>20</v>
@@ -12826,7 +12844,7 @@
     </row>
     <row r="148" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A148" s="1">
-        <v>46143.824305555558</v>
+        <v>46132.854826388888</v>
       </c>
       <c r="B148">
         <v>20</v>
@@ -12885,7 +12903,7 @@
     </row>
     <row r="149" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A149" s="1">
-        <v>46144.330555555563</v>
+        <v>46126.927673611113</v>
       </c>
       <c r="B149">
         <v>23</v>
@@ -12944,7 +12962,7 @@
     </row>
     <row r="150" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A150" s="1">
-        <v>46144.59652777778</v>
+        <v>46127.124594907407</v>
       </c>
       <c r="B150">
         <v>21</v>
@@ -13003,7 +13021,7 @@
     </row>
     <row r="151" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A151" s="1">
-        <v>46144.7</v>
+        <v>46130.326817129629</v>
       </c>
       <c r="B151">
         <v>22</v>
@@ -13062,7 +13080,7 @@
     </row>
     <row r="152" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A152" s="1">
-        <v>46144.888194444437</v>
+        <v>46125.448518518519</v>
       </c>
       <c r="B152">
         <v>20</v>
@@ -13121,7 +13139,7 @@
     </row>
     <row r="153" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A153" s="1">
-        <v>46145.299305555563</v>
+        <v>46130.278391203705</v>
       </c>
       <c r="B153">
         <v>20</v>
@@ -13180,7 +13198,7 @@
     </row>
     <row r="154" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A154" s="1">
-        <v>46145.489583333343</v>
+        <v>46125.492048611108</v>
       </c>
       <c r="B154">
         <v>20</v>
@@ -13239,7 +13257,7 @@
     </row>
     <row r="155" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A155" s="1">
-        <v>46145.537499999999</v>
+        <v>46131.935347222221</v>
       </c>
       <c r="B155">
         <v>21</v>
@@ -13298,7 +13316,7 @@
     </row>
     <row r="156" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A156" s="1">
-        <v>46145.770138888889</v>
+        <v>46131.260648148149</v>
       </c>
       <c r="B156">
         <v>18</v>
@@ -13357,7 +13375,7 @@
     </row>
     <row r="157" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A157" s="1">
-        <v>46145.886111111111</v>
+        <v>46131.273761574077</v>
       </c>
       <c r="B157">
         <v>18</v>
@@ -13416,7 +13434,7 @@
     </row>
     <row r="158" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A158" s="1">
-        <v>46146.313888888893</v>
+        <v>46130.321145833332</v>
       </c>
       <c r="B158">
         <v>20</v>
@@ -13475,7 +13493,7 @@
     </row>
     <row r="159" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A159" s="1">
-        <v>46146.540277777778</v>
+        <v>46130.106620370374</v>
       </c>
       <c r="B159">
         <v>21</v>
@@ -13534,7 +13552,7 @@
     </row>
     <row r="160" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A160" s="1">
-        <v>46146.620833333327</v>
+        <v>46132.657986111109</v>
       </c>
       <c r="B160">
         <v>20</v>
@@ -13593,7 +13611,7 @@
     </row>
     <row r="161" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A161" s="1">
-        <v>46146.685416666667</v>
+        <v>46128.673217592594</v>
       </c>
       <c r="B161">
         <v>19</v>
@@ -13652,7 +13670,7 @@
     </row>
     <row r="162" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A162" s="1">
-        <v>46146.828472222223</v>
+        <v>46132.758506944447</v>
       </c>
       <c r="B162">
         <v>20</v>
@@ -13711,7 +13729,7 @@
     </row>
     <row r="163" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A163" s="1">
-        <v>46147.298611111109</v>
+        <v>46127.838854166665</v>
       </c>
       <c r="B163">
         <v>20</v>
@@ -13770,7 +13788,7 @@
     </row>
     <row r="164" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A164" s="1">
-        <v>46147.500694444447</v>
+        <v>46129.866493055553</v>
       </c>
       <c r="B164">
         <v>19</v>
@@ -13829,7 +13847,7 @@
     </row>
     <row r="165" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A165" s="1">
-        <v>46147.787499999999</v>
+        <v>46126.62122685185</v>
       </c>
       <c r="B165">
         <v>20</v>
@@ -13888,7 +13906,7 @@
     </row>
     <row r="166" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A166" s="1">
-        <v>46148.318055555559</v>
+        <v>46133.335092592592</v>
       </c>
       <c r="B166">
         <v>18</v>
@@ -13947,7 +13965,7 @@
     </row>
     <row r="167" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A167" s="1">
-        <v>46148.443055555559</v>
+        <v>46129.446203703701</v>
       </c>
       <c r="B167">
         <v>28</v>
@@ -14006,7 +14024,7 @@
     </row>
     <row r="168" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A168" s="1">
-        <v>46148.627083333333</v>
+        <v>46127.036840277775</v>
       </c>
       <c r="B168">
         <v>19</v>
@@ -14065,7 +14083,7 @@
     </row>
     <row r="169" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A169" s="1">
-        <v>46148.643750000003</v>
+        <v>46125.137349537035</v>
       </c>
       <c r="B169">
         <v>22</v>
@@ -14124,7 +14142,7 @@
     </row>
     <row r="170" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A170" s="1">
-        <v>46148.693749999999</v>
+        <v>46133.878831018519</v>
       </c>
       <c r="B170">
         <v>18</v>
@@ -14183,7 +14201,7 @@
     </row>
     <row r="171" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A171" s="1">
-        <v>46148.832638888889</v>
+        <v>46130.874907407408</v>
       </c>
       <c r="B171">
         <v>19</v>
@@ -14242,7 +14260,7 @@
     </row>
     <row r="172" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A172" s="1">
-        <v>46148.95208333333</v>
+        <v>46133.778032407405</v>
       </c>
       <c r="B172">
         <v>19</v>
@@ -14301,7 +14319,7 @@
     </row>
     <row r="173" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A173" s="1">
-        <v>46149.293749999997</v>
+        <v>46132.829594907409</v>
       </c>
       <c r="B173">
         <v>23</v>
@@ -14360,7 +14378,7 @@
     </row>
     <row r="174" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A174" s="1">
-        <v>46149.38958333333</v>
+        <v>46132.396562499998</v>
       </c>
       <c r="B174">
         <v>21</v>
@@ -14419,7 +14437,7 @@
     </row>
     <row r="175" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A175" s="1">
-        <v>46149.601388888892</v>
+        <v>46130.082048611112</v>
       </c>
       <c r="B175">
         <v>30</v>
@@ -14478,7 +14496,7 @@
     </row>
     <row r="176" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A176" s="1">
-        <v>46149.63958333333</v>
+        <v>46126.855300925927</v>
       </c>
       <c r="B176">
         <v>19</v>
@@ -14537,7 +14555,7 @@
     </row>
     <row r="177" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A177" s="1">
-        <v>46149.679861111108</v>
+        <v>46128.626319444447</v>
       </c>
       <c r="B177">
         <v>22</v>
@@ -14596,7 +14614,7 @@
     </row>
     <row r="178" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A178" s="1">
-        <v>46149.95</v>
+        <v>46129.59883101852</v>
       </c>
       <c r="B178">
         <v>19</v>
@@ -14655,7 +14673,7 @@
     </row>
     <row r="179" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A179" s="1">
-        <v>46150.327777777777</v>
+        <v>46130.122083333335</v>
       </c>
       <c r="B179">
         <v>21</v>
@@ -14714,7 +14732,7 @@
     </row>
     <row r="180" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A180" s="1">
-        <v>46150.362500000003</v>
+        <v>46127.681967592594</v>
       </c>
       <c r="B180">
         <v>20</v>
@@ -14773,7 +14791,7 @@
     </row>
     <row r="181" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A181" s="1">
-        <v>46150.643055555563</v>
+        <v>46126.019513888888</v>
       </c>
       <c r="B181">
         <v>24</v>
@@ -14832,7 +14850,7 @@
     </row>
     <row r="182" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A182" s="1">
-        <v>46150.842361111107</v>
+        <v>46133.6565625</v>
       </c>
       <c r="B182">
         <v>19</v>
@@ -14891,7 +14909,7 @@
     </row>
     <row r="183" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A183" s="1">
-        <v>46151.297222222223</v>
+        <v>46128.762499999997</v>
       </c>
       <c r="B183">
         <v>21</v>
@@ -14950,7 +14968,7 @@
     </row>
     <row r="184" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A184" s="1">
-        <v>46151.352777777778</v>
+        <v>46131.817280092589</v>
       </c>
       <c r="B184">
         <v>24</v>
@@ -15009,7 +15027,7 @@
     </row>
     <row r="185" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A185" s="1">
-        <v>46151.597222222219</v>
+        <v>46133.731423611112</v>
       </c>
       <c r="B185">
         <v>22</v>
@@ -15068,7 +15086,7 @@
     </row>
     <row r="186" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A186" s="1">
-        <v>46151.776388888888</v>
+        <v>46126.33021990741</v>
       </c>
       <c r="B186">
         <v>20</v>
@@ -15127,7 +15145,7 @@
     </row>
     <row r="187" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A187" s="1">
-        <v>46152.344444444447</v>
+        <v>46133.320729166669</v>
       </c>
       <c r="B187">
         <v>20</v>
@@ -15139,7 +15157,7 @@
         <v>34</v>
       </c>
       <c r="E187" t="s">
-        <v>80</v>
+        <v>21</v>
       </c>
       <c r="F187" t="s">
         <v>55</v>
@@ -15186,7 +15204,7 @@
     </row>
     <row r="188" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A188" s="1">
-        <v>46152.542361111111</v>
+        <v>46130.659247685187</v>
       </c>
       <c r="B188">
         <v>21</v>
@@ -15198,7 +15216,7 @@
         <v>34</v>
       </c>
       <c r="E188" t="s">
-        <v>35</v>
+        <v>21</v>
       </c>
       <c r="F188" t="s">
         <v>22</v>
@@ -15245,7 +15263,7 @@
     </row>
     <row r="189" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A189" s="1">
-        <v>46152.768055555563</v>
+        <v>46130.995416666665</v>
       </c>
       <c r="B189">
         <v>22</v>
@@ -15257,7 +15275,7 @@
         <v>20</v>
       </c>
       <c r="E189" t="s">
-        <v>285</v>
+        <v>21</v>
       </c>
       <c r="F189" t="s">
         <v>55</v>
@@ -15304,7 +15322,7 @@
     </row>
     <row r="190" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A190" s="1">
-        <v>46152.928472222222</v>
+        <v>46126.236168981479</v>
       </c>
       <c r="B190">
         <v>19</v>
@@ -15363,7 +15381,7 @@
     </row>
     <row r="191" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A191" s="1">
-        <v>46153.332638888889</v>
+        <v>46128.480740740742</v>
       </c>
       <c r="B191">
         <v>21</v>
@@ -15422,7 +15440,7 @@
     </row>
     <row r="192" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A192" s="1">
-        <v>46153.534722222219</v>
+        <v>46130.165300925924</v>
       </c>
       <c r="B192">
         <v>20</v>
@@ -15481,7 +15499,7 @@
     </row>
     <row r="193" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A193" s="1">
-        <v>46153.813194444447</v>
+        <v>46130.451979166668</v>
       </c>
       <c r="B193">
         <v>19</v>
@@ -15493,7 +15511,7 @@
         <v>135</v>
       </c>
       <c r="E193" t="s">
-        <v>185</v>
+        <v>21</v>
       </c>
       <c r="F193" t="s">
         <v>22</v>
@@ -15540,7 +15558,7 @@
     </row>
     <row r="194" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A194" s="1">
-        <v>46154.322222222218</v>
+        <v>46130.89508101852</v>
       </c>
       <c r="B194">
         <v>22</v>
@@ -15599,7 +15617,7 @@
     </row>
     <row r="195" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A195" s="1">
-        <v>46154.40347222222</v>
+        <v>46133.959976851853</v>
       </c>
       <c r="B195">
         <v>20</v>
@@ -15658,7 +15676,7 @@
     </row>
     <row r="196" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A196" s="1">
-        <v>46154.667361111111</v>
+        <v>46130.34578703704</v>
       </c>
       <c r="B196">
         <v>19</v>
@@ -15717,7 +15735,7 @@
     </row>
     <row r="197" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A197" s="1">
-        <v>46154.788194444453</v>
+        <v>46131.788171296299</v>
       </c>
       <c r="B197">
         <v>20</v>
@@ -15729,7 +15747,7 @@
         <v>34</v>
       </c>
       <c r="E197" t="s">
-        <v>163</v>
+        <v>21</v>
       </c>
       <c r="F197" t="s">
         <v>55</v>
@@ -15776,7 +15794,7 @@
     </row>
     <row r="198" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A198" s="1">
-        <v>46154.94027777778</v>
+        <v>46131.109571759262</v>
       </c>
       <c r="B198">
         <v>19</v>
@@ -15835,7 +15853,7 @@
     </row>
     <row r="199" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A199" s="1">
-        <v>46155.320138888892</v>
+        <v>46133.686736111114</v>
       </c>
       <c r="B199">
         <v>19</v>
@@ -15847,7 +15865,7 @@
         <v>20</v>
       </c>
       <c r="E199" t="s">
-        <v>285</v>
+        <v>21</v>
       </c>
       <c r="F199" t="s">
         <v>55</v>
@@ -15894,7 +15912,7 @@
     </row>
     <row r="200" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A200" s="1">
-        <v>46155.463194444441</v>
+        <v>46133.098703703705</v>
       </c>
       <c r="B200">
         <v>19</v>
@@ -15953,7 +15971,7 @@
     </row>
     <row r="201" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A201" s="1">
-        <v>46155.629166666673</v>
+        <v>46129.784178240741</v>
       </c>
       <c r="B201">
         <v>25</v>

</xml_diff>